<commit_message>
feat: organize active stage render field
</commit_message>
<xml_diff>
--- a/BlackStage_OS_Development_Tracker.xlsx
+++ b/BlackStage_OS_Development_Tracker.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="116">
   <si>
     <t>Updated 2026-05-14. Repo-backed tracker reflects current Stage Shell, render-field, and live-harness evidence.</t>
   </si>
@@ -307,6 +307,63 @@
   </si>
   <si>
     <t>Planned</t>
+  </si>
+  <si>
+    <t>Updated 2026-05-14. Repo-backed tracker reflects current Stage Shell, Browser validation, render-field, and live-harness evidence.</t>
+  </si>
+  <si>
+    <t>Render organization intelligence v1</t>
+  </si>
+  <si>
+    <t>Taste-review active render field after voice pass</t>
+  </si>
+  <si>
+    <t>Use Browser plugin for manual visual QA</t>
+  </si>
+  <si>
+    <t>Render organization intelligence v1 added; Browser-plugin visual QA still needs Cheick taste review.</t>
+  </si>
+  <si>
+    <t>LOG-004</t>
+  </si>
+  <si>
+    <t>Render organization intelligence pass</t>
+  </si>
+  <si>
+    <t>Primary plan display, topology strip, cleaner command rail, and short-viewport collision handling.</t>
+  </si>
+  <si>
+    <t>First Browser screenshot exposed crowding; second pass hid secondary chrome in shallow viewport.</t>
+  </si>
+  <si>
+    <t>Cheick flagged lack of organization intelligence and display quality.</t>
+  </si>
+  <si>
+    <t>Hierarchy has to be legible before live tool use feels magical.</t>
+  </si>
+  <si>
+    <t>Browser-plugin validation catches compact-surface overlap missed by large screenshots.</t>
+  </si>
+  <si>
+    <t>DEC-005</t>
+  </si>
+  <si>
+    <t>Validation</t>
+  </si>
+  <si>
+    <t>Manual rendered QA should use the Browser plugin before standalone Playwright fallback.</t>
+  </si>
+  <si>
+    <t>Cheick explicitly requested Browser for testing rendered local UI.</t>
+  </si>
+  <si>
+    <t>Standalone Playwright only; Browser-first visual QA</t>
+  </si>
+  <si>
+    <t>docs/research/runs/2026-05-14-render-organization-intelligence-slice.md</t>
+  </si>
+  <si>
+    <t>Render organization intelligence v1 added; Cheick taste review remains open.</t>
   </si>
 </sst>
 </file>
@@ -944,7 +1001,7 @@
     </row>
     <row r="2">
       <c r="A2" s="22" t="s">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="B2" t="str"/>
       <c r="C2" t="str"/>
@@ -1115,7 +1172,7 @@
     </row>
     <row r="15">
       <c r="A15" s="26" t="s">
-        <v>9</v>
+        <v>98</v>
       </c>
       <c r="B15" s="26" t="s">
         <v>10</v>
@@ -1148,7 +1205,7 @@
     </row>
     <row r="18">
       <c r="A18" s="26" t="s">
-        <v>15</v>
+        <v>99</v>
       </c>
       <c r="B18" s="26" t="s">
         <v>12</v>
@@ -1159,24 +1216,24 @@
     </row>
     <row r="19">
       <c r="A19" s="26" t="s">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="B19" s="26" t="s">
         <v>10</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="26" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" s="26" t="s">
         <v>10</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2204,7 +2261,7 @@
         <v>Screenshots show idle, working, approval, artifact states.</v>
       </c>
       <c r="I19" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="J19" t="str">
         <v>Yes</v>
@@ -2620,6 +2677,38 @@
         <v>39</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H5" t="s">
+        <v>106</v>
+      </c>
+      <c r="I5" t="s">
+        <v>107</v>
+      </c>
+      <c r="J5" t="s">
+        <v>108</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" sqref="C2:C100">
@@ -2808,6 +2897,38 @@
         <v>54</v>
       </c>
       <c r="J5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" t="s">
+        <v>112</v>
+      </c>
+      <c r="H6" t="s">
+        <v>113</v>
+      </c>
+      <c r="I6" t="s">
+        <v>114</v>
+      </c>
+      <c r="J6" t="s">
         <v>48</v>
       </c>
     </row>
@@ -3256,7 +3377,7 @@
       </c>
       <c r="E8" t="str"/>
       <c r="F8" t="s">
-        <v>61</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Build cinematic stage render manifest
</commit_message>
<xml_diff>
--- a/BlackStage_OS_Development_Tracker.xlsx
+++ b/BlackStage_OS_Development_Tracker.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
   <si>
     <t>Updated 2026-05-14. Repo-backed tracker reflects current Stage Shell, render-field, and live-harness evidence.</t>
   </si>
@@ -364,6 +364,147 @@
   </si>
   <si>
     <t>Render organization intelligence v1 added; Cheick taste review remains open.</t>
+  </si>
+  <si>
+    <t>Updated 2026-05-14. Repo-backed tracker now includes cinematic render-system study, StageSceneManifest contract, Browser-first visual QA, and live-harness evidence.</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Cinematic render system Phase 1</t>
+  </si>
+  <si>
+    <t>Codex</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>BS-019</t>
+  </si>
+  <si>
+    <t>Stage Rendering</t>
+  </si>
+  <si>
+    <t>1 Stage Shell v0</t>
+  </si>
+  <si>
+    <t>Create cinematic scene manifest and fluid vector renderer</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>P0</t>
+  </si>
+  <si>
+    <t>Codex</t>
+  </si>
+  <si>
+    <t>IntentThread compiles to scene manifest; UI renders semantic roles, edges, and liquid field without dashboard feel.</t>
+  </si>
+  <si>
+    <t>stage-core/stage-web typecheck; Browser-plugin screenshot; e2e visual assertions.</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>BS-003, BS-008, BS-018</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Manifest contract started from video/json-render study; Phase 1 vector field next.</t>
+  </si>
+  <si>
+    <t>LOG-005</t>
+  </si>
+  <si>
+    <t>2026-05-14</t>
+  </si>
+  <si>
+    <t>UX/Research</t>
+  </si>
+  <si>
+    <t>BS-019</t>
+  </si>
+  <si>
+    <t>Study cinematic demo video and json-render prior art</t>
+  </si>
+  <si>
+    <t>Extracted video frames, inspected json-render, and added StageSceneManifest contract.</t>
+  </si>
+  <si>
+    <t>No live aesthetic validation yet; next slice must prove the vector field visually.</t>
+  </si>
+  <si>
+    <t>Cheick supplied target video and called current display not good enough.</t>
+  </si>
+  <si>
+    <t>The target is a cognitive scene system, not prettier cards.</t>
+  </si>
+  <si>
+    <t>Borrow guarded specs and patch streams from json-render, but render scene semantics.</t>
+  </si>
+  <si>
+    <t>docs/research/runs/2026-05-14-cinematic-render-system-study.md</t>
+  </si>
+  <si>
+    <t>Build StageSceneField vector layer and Browser screenshot gate.</t>
+  </si>
+  <si>
+    <t>DEC-006</t>
+  </si>
+  <si>
+    <t>2026-05-14</t>
+  </si>
+  <si>
+    <t>Rendering</t>
+  </si>
+  <si>
+    <t>Blackstage render system will use a guarded scene manifest and patch stream, not arbitrary generated UI or static cards.</t>
+  </si>
+  <si>
+    <t>Accepted</t>
+  </si>
+  <si>
+    <t>Cheick + Codex</t>
+  </si>
+  <si>
+    <t>The video target requires cinematic scene semantics while preserving replayability and approval safety.</t>
+  </si>
+  <si>
+    <t>Static CSS cards; arbitrary agent DOM; json-render component tree; Blackstage scene graph.</t>
+  </si>
+  <si>
+    <t>docs/28_cinematic_rendering_system.md</t>
+  </si>
+  <si>
+    <t>2026-05-21</t>
+  </si>
+  <si>
+    <t>Inspired by json-render contracts, adapted for camera, substrate, material, motion, clusters, and edges.</t>
+  </si>
+  <si>
+    <t>Orb-first idle, scene manifest contract, and spatial render field; continue vector-field and taste QA after live sessions.</t>
+  </si>
+  <si>
+    <t>StageSceneManifest moves taste-critical organization into code; Browser-plugin visual QA remains the gate.</t>
   </si>
 </sst>
 </file>
@@ -705,7 +846,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BacklogTable" displayName="BacklogTable" ref="A1:N19" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BacklogTable" displayName="BacklogTable" ref="A1:N21" headerRowCount="1">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Workstream"/>
@@ -976,7 +1117,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="52" hidden="0" customWidth="1"/>
@@ -1001,7 +1142,7 @@
     </row>
     <row r="2">
       <c r="A2" s="22" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="B2" t="str"/>
       <c r="C2" t="str"/>
@@ -1035,8 +1176,8 @@
       <c r="A5" s="26" t="str">
         <v>Backlog Tasks</v>
       </c>
-      <c r="B5" s="26">
-        <v>18</v>
+      <c r="B5" s="26" t="str">
+        <v>20</v>
       </c>
       <c r="C5" s="26" t="str">
         <v>Total initial tasks</v>
@@ -1047,16 +1188,16 @@
       <c r="F5" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="G5" s="26">
-        <v>15</v>
+      <c r="G5" s="26" t="str">
+        <v>16</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="str">
         <v>Done Tasks</v>
       </c>
-      <c r="B6" s="26">
-        <v>15</v>
+      <c r="B6" s="26" t="str">
+        <v>16</v>
       </c>
       <c r="C6" s="26" t="str">
         <v>Completed items</v>
@@ -1075,8 +1216,8 @@
       <c r="A7" s="26" t="str">
         <v>In Progress Tasks</v>
       </c>
-      <c r="B7" s="26">
-        <v>3</v>
+      <c r="B7" s="26" t="s">
+        <v>118</v>
       </c>
       <c r="C7" s="26" t="str">
         <v>Active work</v>
@@ -1087,16 +1228,16 @@
       <c r="F7" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="G7" s="26">
-        <v>0</v>
+      <c r="G7" s="26" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="26" t="str">
         <v>P0 Tasks</v>
       </c>
-      <c r="B8" s="26">
-        <v>13</v>
+      <c r="B8" s="26" t="s">
+        <v>119</v>
       </c>
       <c r="C8" s="26" t="str">
         <v>Critical path</v>
@@ -1171,14 +1312,14 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="26" t="s">
-        <v>98</v>
+      <c r="A15" s="26" t="str">
+        <v>Build StageSceneField vector layer and live voice debug overlay</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" s="26" t="s">
-        <v>1</v>
+        <v>122</v>
+      </c>
+      <c r="C15" s="26" t="str">
+        <v>In Progress</v>
       </c>
     </row>
     <row r="16">
@@ -1242,7 +1383,7 @@
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="R88fb916a896f4ef7"/>
+  <drawing ns1:id="R88fb916a896f4ef7"/>
 </worksheet>
 </file>
 
@@ -1528,7 +1669,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" hidden="0" customWidth="1"/>
@@ -2272,6 +2413,90 @@
       <c r="L19" t="str"/>
       <c r="M19" t="str"/>
       <c r="N19" t="str"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>124</v>
+      </c>
+      <c r="B20" t="s">
+        <v>125</v>
+      </c>
+      <c r="C20" t="s">
+        <v>126</v>
+      </c>
+      <c r="D20" t="s">
+        <v>127</v>
+      </c>
+      <c r="E20" t="s">
+        <v>128</v>
+      </c>
+      <c r="F20" t="s">
+        <v>129</v>
+      </c>
+      <c r="G20" t="s">
+        <v>130</v>
+      </c>
+      <c r="H20" t="s">
+        <v>131</v>
+      </c>
+      <c r="I20" t="s">
+        <v>132</v>
+      </c>
+      <c r="J20" t="s">
+        <v>133</v>
+      </c>
+      <c r="K20" t="s">
+        <v>134</v>
+      </c>
+      <c r="L20" t="s">
+        <v>135</v>
+      </c>
+      <c r="M20" t="s">
+        <v>136</v>
+      </c>
+      <c r="N20" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>BS-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Stage Frontend</v>
+      </c>
+      <c r="C21" t="str">
+        <v>1 Stage Shell v0</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Browser compact render QA and orb voice entry</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Done</v>
+      </c>
+      <c r="F21" t="str">
+        <v>P0</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Codex</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Browser in-app compact viewport keeps active stage regions separated and live voice/debug controls reachable.</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Browser plugin geometry check reports zero overlaps and visible Speak/Export controls.</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K21" t="str">
+        <v>BS-018, BS-019</v>
+      </c>
+      <c r="L21" t="str"/>
+      <c r="M21" t="str"/>
+      <c r="N21" t="str">
+        <v>Logged in 2026-05-15 browser compact render slice.</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E19">
@@ -2300,7 +2525,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R281c859479774d5c"/>
+    <tablePart ns1:id="R281c859479774d5c"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2534,7 +2759,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" hidden="0" customWidth="1"/>
@@ -2709,6 +2934,82 @@
         <v>108</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C6" t="s">
+        <v>140</v>
+      </c>
+      <c r="D6" t="s">
+        <v>141</v>
+      </c>
+      <c r="E6" t="s">
+        <v>142</v>
+      </c>
+      <c r="F6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G6" t="s">
+        <v>144</v>
+      </c>
+      <c r="H6" t="s">
+        <v>145</v>
+      </c>
+      <c r="I6" t="s">
+        <v>146</v>
+      </c>
+      <c r="J6" t="s">
+        <v>147</v>
+      </c>
+      <c r="K6" t="s">
+        <v>148</v>
+      </c>
+      <c r="L6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>LOG-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-05-15</v>
+      </c>
+      <c r="C7" t="str">
+        <v>UX/Validation</v>
+      </c>
+      <c r="D7" t="str">
+        <v>BS-020</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Browser compact render and orb entry QA</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Idle orb is demo-free; compact active field keeps intent, plan, evidence, labor, approval, artifact, command, and research zones separated.</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Initial compact pass hid command/debug; focused dock then overlapped the document object before the one-row compact fix.</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Cheick explicitly corrected tool choice to Browser plugin.</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Quiet chrome must stay reachable; hidden controls cannot block live testing.</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Browser plugin catches real in-app viewport issues that headless gates can miss.</v>
+      </c>
+      <c r="K7" t="str">
+        <v>docs/research/runs/2026-05-15-browser-compact-render-and-orb-entry-slice.md</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Continue StageSceneField vector layer and live voice debug QA.</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" sqref="C2:C100">
@@ -2717,13 +3018,13 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="Rdb356ef7547d4528"/>
+    <tablePart ns1:id="Rdb356ef7547d4528"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" hidden="0" customWidth="1"/>
@@ -2932,6 +3233,76 @@
         <v>48</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>150</v>
+      </c>
+      <c r="B7" t="s">
+        <v>151</v>
+      </c>
+      <c r="C7" t="s">
+        <v>152</v>
+      </c>
+      <c r="D7" t="s">
+        <v>153</v>
+      </c>
+      <c r="E7" t="s">
+        <v>154</v>
+      </c>
+      <c r="F7" t="s">
+        <v>155</v>
+      </c>
+      <c r="G7" t="s">
+        <v>156</v>
+      </c>
+      <c r="H7" t="s">
+        <v>157</v>
+      </c>
+      <c r="I7" t="s">
+        <v>158</v>
+      </c>
+      <c r="J7" t="s">
+        <v>159</v>
+      </c>
+      <c r="K7" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>DEC-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-05-15</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Rendering</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Compact active sessions must keep voice and debug entrypoints reachable instead of hiding them completely.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Accepted</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Cheick + Codex</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Live testing depends on visible Speak and debug export controls even when the field is intentionally quiet.</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Hide all chrome; always show full panels; compact one-row command and trace controls</v>
+      </c>
+      <c r="I8" t="str">
+        <v>docs/research/runs/2026-05-15-browser-compact-render-and-orb-entry-slice.md</v>
+      </c>
+      <c r="J8" t="str">
+        <v>2026-05-22</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Browser plugin geometry check is the acceptance gate for compact active sessions.</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation type="list" sqref="C2:C100">
@@ -2943,13 +3314,13 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="Rb9393f6f1d2545c7"/>
+    <tablePart ns1:id="Rb9393f6f1d2545c7"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" hidden="0" customWidth="1"/>
@@ -3020,7 +3391,7 @@
         <v>Kills category thesis.</v>
       </c>
       <c r="G2" t="s">
-        <v>88</v>
+        <v>161</v>
       </c>
       <c r="H2" t="str">
         <v>Cheick</v>
@@ -3185,7 +3556,7 @@
         <v>Product becomes undifferentiated.</v>
       </c>
       <c r="G7" t="s">
-        <v>94</v>
+        <v>162</v>
       </c>
       <c r="H7" t="str">
         <v>GPT-5.5 Pro</v>
@@ -3217,7 +3588,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="R5cf31a07ae2a4736"/>
+    <tablePart ns1:id="R5cf31a07ae2a4736"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Build cinematic stage scene field
</commit_message>
<xml_diff>
--- a/BlackStage_OS_Development_Tracker.xlsx
+++ b/BlackStage_OS_Development_Tracker.xlsx
@@ -2498,6 +2498,150 @@
         <v>Logged in 2026-05-15 browser compact render slice.</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BS-021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Stage Rendering</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1 Stage Shell v0</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Make render field the goal center: semantic stage coordinates and focal floor</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Active field uses scene coordinates, a focal floor/horizon, hidden QA deep links, and Browser evidence without visible demo buttons.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Browser desktop/mobile visual QA; typecheck/lint/build/test</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>BS-019, BS-020</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Next: central approval ritual and geometric agent labor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BS-022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Stage Rendering</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1 Stage Shell v0</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Turn approval and agent labor into central cinematic scene objects</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Pending approvals dim the field and become central ritual objects; agent labor can expand from geometry into audit feed.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Browser visual QA plus e2e scene-manifest assertions</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>BS-021</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Reference video frames show approval/action and labor geometry as the next gap.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E19">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -3010,6 +3154,130 @@
         <v>Continue StageSceneField vector layer and live voice debug QA.</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LOG-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UX/Research</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BS-021</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Frame-by-frame render field reference analysis</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Extracted all 192 frames and translated the video into stage, focal, approval, and labor requirements.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Confirmed prior UI still leaned too much toward cards/dashboard composition.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Cheick supplied a second cinematic reference and redirected the goal toward rendering field animation.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>One focal object plus orbiting support reads smarter than many equal panels.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Frame sampling turned taste feedback into concrete renderer requirements.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>docs/research/runs/2026-05-15-render-field-reference-analysis.md</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Build central approval ritual and geometric labor field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LOG-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>UX/Build</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BS-021</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Semantic stage-coordinate render pass</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>StageSceneManifest now drives x/y/depth/scale; StageSceneField draws focal floor and horizon; Browser QA shows no active-field overlaps.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Browser input path exposed clipboard limitations, so hidden scenario/instant QA links were added.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>None beyond Cheick's rendering-first correction.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>The field must own organization; CSS grid placement is not enough.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Browser visual checks need deterministic deep links that do not pollute startup UX.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>docs/research/runs/2026-05-15-stage-scene-field-vector-slice.md</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Make approval and labor materialize as central scene states.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" sqref="C2:C100">
@@ -3301,6 +3569,120 @@
       </c>
       <c r="K8" t="str">
         <v>Browser plugin geometry check is the acceptance gate for compact active sessions.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DEC-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Rendering</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>The active goal is rendering-first until the field itself feels like organized intelligence.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Cheick + Codex</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>The project thesis fails if runtime features work but the surface still reads like a dark dashboard.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Continue backend/runtime first; polish cards; render-field-first goal amendment.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>codex/goals/first_long_run_stage_shell_v0_after_prompt1.md</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Reference video 2 is now a north-star artifact for stage composition and motion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DEC-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Use hidden deep-link QA parameters for visual scenarios instead of visible demo buttons.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>The startup UX must remain one orb and one instruction while Browser QA still needs deterministic active states.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Visible demo buttons; manual typing only; hidden query controls.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>docs/28_cinematic_rendering_system.md</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Supported query controls: stageScenario, stageIntent, stageInstant, stageDelayMultiplier.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add render field zone flow
</commit_message>
<xml_diff>
--- a/BlackStage_OS_Development_Tracker.xlsx
+++ b/BlackStage_OS_Development_Tracker.xlsx
@@ -846,7 +846,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BacklogTable" displayName="BacklogTable" ref="A1:N21" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BacklogTable" displayName="BacklogTable" ref="A1:N24" headerRowCount="1">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Workstream"/>
@@ -2642,6 +2642,78 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BS-023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Stage Rendering</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1 Stage Shell v0</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Add semantic render zones and flow spine</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>StageSceneManifest emits active zones; StageSceneField renders zone bands/flow; approved desktop scenes keep objects and command dock clear.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Browser desktop geometry QA and targeted e2e overlap gate pass.</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>BS-021, BS-022</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Browser found approved-scene overlap; anchors and zone grammar were retuned. Next: central approval ritual.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E19">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -3278,6 +3350,68 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LOG-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>UX/Build</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BS-023</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Render zone flow and overlap hardening</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Added semantic scene zones, zone-flow spine, retuned anchors, and e2e geometry checks for approved scenes.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Browser desktop QA exposed focal-plan overlap from secondary task/model objects before the retune.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Cheick asked to continue systematically toward the reality-interface goal.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>The field needs a visible grammar, not only better object coordinates.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Browser geometry turns taste feedback into deterministic renderer work.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>docs/research/runs/2026-05-16-render-zone-flow-slice.md</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Make approval and visible labor feel central instead of rail-shaped.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" sqref="C2:C100">
@@ -3682,6 +3816,63 @@
       <c r="K10" t="inlineStr">
         <is>
           <t>Supported query controls: stageScenario, stageIntent, stageInstant, stageDelayMultiplier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DEC-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Rendering</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Render organization belongs in semantic zones plus measured geometry gates, not only CSS placement.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>The user must feel the field organizing intelligence before reading individual cards.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Card coordinates only; semantic zones; full physics engine.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>docs/research/runs/2026-05-16-render-zone-flow-slice.md</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>The next renderer target is central approval and labor geometry.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bind approvals to focused stage objects
</commit_message>
<xml_diff>
--- a/BlackStage_OS_Development_Tracker.xlsx
+++ b/BlackStage_OS_Development_Tracker.xlsx
@@ -846,7 +846,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BacklogTable" displayName="BacklogTable" ref="A1:N25" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BacklogTable" displayName="BacklogTable" ref="A1:N26" headerRowCount="1">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Workstream"/>
@@ -2786,6 +2786,78 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="inlineStr">
+        <x:is>
+          <x:t>BS-025</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" t="inlineStr">
+        <x:is>
+          <x:t>Stage Rendering</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" t="inlineStr">
+        <x:is>
+          <x:t>1 Stage Shell v0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D26" t="inlineStr">
+        <x:is>
+          <x:t>Bind pending approval to focused work object</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E26" t="inlineStr">
+        <x:is>
+          <x:t>Done</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F26" t="inlineStr">
+        <x:is>
+          <x:t>P0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G26" t="inlineStr">
+        <x:is>
+          <x:t>Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H26" t="inlineStr">
+        <x:is>
+          <x:t>Pending approval derives one focus object, dims surrounding objects, and draws a visible tether from object to approval threshold.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I26" t="inlineStr">
+        <x:is>
+          <x:t>Browser plugin QA plus e2e confirm one focus object, dimmed non-focus opacity, tether presence, and no threshold overlap.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J26" t="inlineStr">
+        <x:is>
+          <x:t>Yes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K26" t="inlineStr">
+        <x:is>
+          <x:t>BS-024</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L26" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="M26" t="inlineStr">
+        <x:is>
+          <x:t>2026-05-16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N26" t="inlineStr">
+        <x:is>
+          <x:t>Makes approval feel like a field/camera event instead of a detached badge.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E2:E19">
     <x:cfRule type="expression" dxfId="0" priority="1">
@@ -3546,6 +3618,68 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="inlineStr">
+        <x:is>
+          <x:t>LOG-011</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" t="inlineStr">
+        <x:is>
+          <x:t>2026-05-16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" t="inlineStr">
+        <x:is>
+          <x:t>UX/Build</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" t="inlineStr">
+        <x:is>
+          <x:t>BS-025</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" t="inlineStr">
+        <x:is>
+          <x:t>Approval focus pull slice</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" t="inlineStr">
+        <x:is>
+          <x:t>Pending approval now focuses the plan object, dims surrounding objects, and draws an approval tether in the field.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" t="inlineStr">
+        <x:is>
+          <x:t>Browser QA caught that animation was overriding dim opacity until the CSS state was hardened and e2e asserted computed opacity.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H12" t="inlineStr">
+        <x:is>
+          <x:t>Cheick kept the goal centered on rendering-field quality rather than accepting backend progress alone.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I12" t="inlineStr">
+        <x:is>
+          <x:t>Approval reads better when it behaves like a camera/focus event tied to the object under review.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J12" t="inlineStr">
+        <x:is>
+          <x:t>Computed-style Browser checks can catch visual cascade bugs that plain DOM presence checks miss.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K12" t="inlineStr">
+        <x:is>
+          <x:t>docs/research/runs/2026-05-16-approval-focus-pull-slice.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L12" t="inlineStr">
+        <x:is>
+          <x:t>Animate a stronger camera focus pull around the approval-bound object.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C2:C100">
@@ -4064,6 +4198,63 @@
       <x:c r="K12" t="inlineStr">
         <x:is>
           <x:t>Revisit when the approval object becomes more immersive.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="inlineStr">
+        <x:is>
+          <x:t>DEC-012</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" t="inlineStr">
+        <x:is>
+          <x:t>2026-05-16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" t="inlineStr">
+        <x:is>
+          <x:t>Rendering</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" t="inlineStr">
+        <x:is>
+          <x:t>Pending approval should derive a single object-bound focus state from replayable thread and scene state.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" t="inlineStr">
+        <x:is>
+          <x:t>Accepted</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" t="inlineStr">
+        <x:is>
+          <x:t>Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" t="inlineStr">
+        <x:is>
+          <x:t>The field should show exactly what object/action is under review without storing separate visual-only approval state.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H13" t="inlineStr">
+        <x:is>
+          <x:t>Detached threshold only; duplicate approval controls in the field; store manual focus state.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I13" t="inlineStr">
+        <x:is>
+          <x:t>docs/05_system_architecture.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J13" t="inlineStr">
+        <x:is>
+          <x:t>2026-05-20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K13" t="inlineStr">
+        <x:is>
+          <x:t>Next review should evaluate whether the focus pull feels cinematic enough.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>